<commit_message>
simulations working, need to add a confusion matrix
</commit_message>
<xml_diff>
--- a/shipClassTests/testResults/SensedComp_GoodSensors_example.xlsx
+++ b/shipClassTests/testResults/SensedComp_GoodSensors_example.xlsx
@@ -626,7 +626,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <v>2</v>
@@ -660,7 +660,7 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>2</v>

</xml_diff>